<commit_message>
Address code-review findings: retention wording, GCP table, sheet generator, cloud pages
Co-authored-by: Isaac <no-reply@databricks.com>
</commit_message>
<xml_diff>
--- a/templates/security-review-questionnaire.xlsx
+++ b/templates/security-review-questionnaire.xlsx
@@ -740,7 +740,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Data inventory ([02](02-what-data-reaches-an-llm.md))</t>
+          <t>Data inventory (02)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Run-as matrix ([06](06-access-control-and-governance.md))</t>
+          <t>Run-as matrix (06)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
@@ -1574,14 +1574,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Use 'Needs confirmation' for items that only a vendor can settle; see notes/open-questions.md.</t>
+          <t>Use 'Needs confirmation' for items that only a vendor can settle.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Questions come from docs/10-security-review-questionnaire.md. Regenerate with scripts/build_questionnaire_sheet.py.</t>
+          <t>Questions come from docs/10-security-review-questionnaire.md in the genie-security-reviews repository.</t>
         </is>
       </c>
     </row>

</xml_diff>